<commit_message>
Update gallery tags/captions with new assignments; hide What I Make section
Rewrite insert_captions.py to match the plain-HTML gallery markup (post
Claude Design bundle conversion) instead of the old escaped-JS format.
Apply new caption/tag assignments from captions.csv, and update the
gallery filter buttons to match the new tag categories (Christmas,
Easter, Valentine's Day, Thanksgiving, Fourth of July, etc). Comment out
the "What I Make" section and its nav link, and simplify the footer CTA
to "Check me out on Instagram."

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/captions.xlsx
+++ b/captions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a25b430bba704e81/Bakery Business/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\code\sprinkle_kindness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{39072059-7D0F-4AE7-89D3-74ACEF626614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5E1B580-3469-4298-819E-53DFA6549B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E6D96BE6-C545-4343-959E-07A4ED72E808}"/>
+    <workbookView xWindow="-24225" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{E6D96BE6-C545-4343-959E-07A4ED72E808}"/>
   </bookViews>
   <sheets>
     <sheet name="captions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="100">
   <si>
     <t>filename</t>
   </si>
@@ -229,18 +229,12 @@
     <t>IMG_9536.webp</t>
   </si>
   <si>
-    <t xml:space="preserve">Holiday </t>
-  </si>
-  <si>
     <t>Occassions</t>
   </si>
   <si>
     <t>Birthday</t>
   </si>
   <si>
-    <t xml:space="preserve">Occassions </t>
-  </si>
-  <si>
     <t xml:space="preserve">Birthday </t>
   </si>
   <si>
@@ -262,18 +256,6 @@
     <t xml:space="preserve">Baby Shower </t>
   </si>
   <si>
-    <t>Get Togethers</t>
-  </si>
-  <si>
-    <t>Holiday</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anniversary </t>
-  </si>
-  <si>
-    <t>Made some filmaker friends these cookies for their film!</t>
-  </si>
-  <si>
     <t>Valentine's Day</t>
   </si>
   <si>
@@ -289,10 +271,55 @@
     <t>Under-the-Sea themed Baby Shower</t>
   </si>
   <si>
-    <t>A friend's baby shower cookies!</t>
-  </si>
-  <si>
     <t>Fourth of July Party</t>
+  </si>
+  <si>
+    <t>Lemon Lavendar Scone</t>
+  </si>
+  <si>
+    <t>Christmas</t>
+  </si>
+  <si>
+    <t>Easter</t>
+  </si>
+  <si>
+    <t>Thanksgiving</t>
+  </si>
+  <si>
+    <t>Fourth of July</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christmas </t>
+  </si>
+  <si>
+    <t>Lemon Raspberry Filled Cake</t>
+  </si>
+  <si>
+    <t>Film set cookies for friends!</t>
+  </si>
+  <si>
+    <t>Bunny in carrot car!</t>
+  </si>
+  <si>
+    <t>Chocolate Orange Cake</t>
+  </si>
+  <si>
+    <t>Fun hamburger shaped cookies!</t>
+  </si>
+  <si>
+    <t>Cinnamon Rolls for any occasion!</t>
+  </si>
+  <si>
+    <t>Baby lamb cookies</t>
+  </si>
+  <si>
+    <t>"Oh boy, it's a BOY!" cookies!</t>
+  </si>
+  <si>
+    <t>Mocha Chocolate Macarons</t>
+  </si>
+  <si>
+    <t>He is Risen!</t>
   </si>
 </sst>
 </file>
@@ -1154,14 +1181,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8D99861-7A43-4D3D-B597-2654C4B439E9}">
   <dimension ref="A1:C67"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.5546875" customWidth="1"/>
-    <col min="2" max="2" width="35.109375" customWidth="1"/>
-    <col min="3" max="3" width="60.33203125" customWidth="1"/>
+    <col min="1" max="1" width="20.5703125" customWidth="1"/>
+    <col min="2" max="2" width="35.140625" customWidth="1"/>
+    <col min="3" max="3" width="60.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1172,559 +1199,589 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
+      <c r="B8" t="s">
+        <v>90</v>
+      </c>
       <c r="C8" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
       <c r="C10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
+      <c r="B11" t="s">
+        <v>93</v>
+      </c>
       <c r="C11" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
+      <c r="B13" t="s">
+        <v>94</v>
+      </c>
       <c r="C13" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
+      <c r="B14" t="s">
+        <v>95</v>
+      </c>
       <c r="C14" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
+      <c r="B19" t="s">
+        <v>84</v>
+      </c>
       <c r="C19" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>28</v>
       </c>
-      <c r="B27" t="s">
-        <v>88</v>
-      </c>
       <c r="C27" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>29</v>
       </c>
       <c r="C28" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>30</v>
       </c>
+      <c r="B29" t="s">
+        <v>82</v>
+      </c>
       <c r="C29" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>33</v>
       </c>
       <c r="C32" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>34</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>35</v>
       </c>
       <c r="C34" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>36</v>
       </c>
+      <c r="B35" t="s">
+        <v>97</v>
+      </c>
       <c r="C35" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>40</v>
       </c>
       <c r="C39" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C40" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>42</v>
       </c>
       <c r="C41" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>43</v>
       </c>
       <c r="C42" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>44</v>
       </c>
       <c r="C43" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>45</v>
       </c>
+      <c r="B44" t="s">
+        <v>98</v>
+      </c>
       <c r="C44" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>46</v>
       </c>
       <c r="C45" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>47</v>
       </c>
       <c r="C46" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>48</v>
       </c>
       <c r="C47" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>49</v>
       </c>
       <c r="C48" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>50</v>
       </c>
       <c r="C49" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>51</v>
       </c>
       <c r="C50" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>52</v>
       </c>
       <c r="C51" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>53</v>
       </c>
       <c r="C52" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>54</v>
       </c>
       <c r="C53" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>55</v>
       </c>
       <c r="C54" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>56</v>
       </c>
+      <c r="B55" t="s">
+        <v>99</v>
+      </c>
       <c r="C55" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>57</v>
       </c>
       <c r="C56" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>58</v>
       </c>
       <c r="C57" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>59</v>
       </c>
       <c r="C58" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>60</v>
       </c>
       <c r="C59" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>61</v>
       </c>
+      <c r="B60" t="s">
+        <v>98</v>
+      </c>
       <c r="C60" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>62</v>
       </c>
       <c r="C61" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>63</v>
       </c>
       <c r="C62" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>64</v>
       </c>
       <c r="C63" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>65</v>
       </c>
       <c r="C64" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>66</v>
       </c>
       <c r="C65" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>67</v>
       </c>
       <c r="C66" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>68</v>
       </c>
       <c r="C67" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>